<commit_message>
remove model version-based discrepancy in error matrix
Error A_PAA_6001_14 had different recommendations (action_context_de/fr) for 2020 and 2020.1.
</commit_message>
<xml_diff>
--- a/Resources/ErrorMatrix_v3.xlsx
+++ b/Resources/ErrorMatrix_v3.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://fjellfuru-my.sharepoint.com/personal/deborah_marcandella_fjellfuru_ch/Documents/fjellfuru_GmbH/VSA/Kommission_Daten_SE/Projekte/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lwiss\Documents\GitHub\vsa-checker-analytics\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="8_{0E6D4AA1-569B-46D7-9DDC-55163537AA9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2B68AAAA-D6C7-4980-B26C-C8C4AC77C734}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{916D71B8-1451-4803-9B2A-E84D7AA067D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1740" yWindow="585" windowWidth="21180" windowHeight="19665" xr2:uid="{17934C0B-DDC6-4116-8244-60783C96A964}"/>
+    <workbookView xWindow="5070" yWindow="5070" windowWidth="46335" windowHeight="15345" xr2:uid="{17934C0B-DDC6-4116-8244-60783C96A964}"/>
   </bookViews>
   <sheets>
     <sheet name="2020_2020.1" sheetId="3" r:id="rId1"/>
@@ -24,7 +24,6 @@
     <definedName name="_Toc213924540" localSheetId="0">'2020_2020.1'!$L$388</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -45,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13012" uniqueCount="990">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13014" uniqueCount="990">
   <si>
     <t>cid</t>
   </si>
@@ -3080,10 +3079,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3437,12 +3432,13 @@
     <col min="1" max="1" width="14.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="46.42578125" customWidth="1"/>
     <col min="5" max="5" width="13.140625" customWidth="1"/>
-    <col min="6" max="6" width="13" customWidth="1"/>
+    <col min="6" max="6" width="18.140625" customWidth="1"/>
     <col min="7" max="7" width="12.85546875" customWidth="1"/>
     <col min="8" max="8" width="23.5703125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="24" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="17.140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="17.140625" customWidth="1"/>
+    <col min="14" max="14" width="17.140625" customWidth="1"/>
+    <col min="15" max="15" width="74.7109375" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="16.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -32716,6 +32712,12 @@
       </c>
       <c r="N638" t="s">
         <v>959</v>
+      </c>
+      <c r="O638" t="s">
+        <v>971</v>
+      </c>
+      <c r="P638" t="s">
+        <v>986</v>
       </c>
     </row>
     <row r="639" spans="1:16">

</xml_diff>